<commit_message>
Board documents file updated
</commit_message>
<xml_diff>
--- a/Documents/Board Observations/Board Statuses.xlsx
+++ b/Documents/Board Observations/Board Statuses.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>S.No</t>
   </si>
@@ -42,6 +42,27 @@
   </si>
   <si>
     <t>Board not powering up properly</t>
+  </si>
+  <si>
+    <t>Board 02</t>
+  </si>
+  <si>
+    <t>Board 03</t>
+  </si>
+  <si>
+    <t>Board 04</t>
+  </si>
+  <si>
+    <t>Board 05</t>
+  </si>
+  <si>
+    <t>Received some response on EtherCAT on this board. No proper connectivity was achieved.</t>
+  </si>
+  <si>
+    <t>Board 06</t>
+  </si>
+  <si>
+    <t>Tested, MCU is fine and binary flashed through Jlink Commander. Stable response over EtherCAT but no scanning in TwinCAT</t>
   </si>
 </sst>
 </file>
@@ -364,7 +385,7 @@
   <cols>
     <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="3" max="3" width="114.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -393,6 +414,9 @@
       <c r="A3">
         <v>2</v>
       </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
       <c r="C3" t="s">
         <v>5</v>
       </c>
@@ -401,26 +425,44 @@
       <c r="A4">
         <v>3</v>
       </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>